<commit_message>
present value discount factored into OBJ; IC sensitivity ongoing
</commit_message>
<xml_diff>
--- a/horizon excursion/15 years - Initial Condition sensitivity/starts/Starting_point.xlsx
+++ b/horizon excursion/15 years - Initial Condition sensitivity/starts/Starting_point.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/horizon excursion/15 years - Initial Condition sensitivity/starts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="563" documentId="13_ncr:1_{30A8FEE2-BE8F-4FE6-A73D-C8D61511F8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40B5B69B-3E62-40D6-916B-8A4FB536AB38}"/>
+  <xr:revisionPtr revIDLastSave="961" documentId="13_ncr:1_{30A8FEE2-BE8F-4FE6-A73D-C8D61511F8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F9E96DB-B215-4E29-9A72-C54969FF6163}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15" yWindow="15" windowWidth="20460" windowHeight="10770" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">I_start!#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Medium_Capacity!$A$2:$P$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Q_start!$A$1:$S$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Q_start!$A$1:$P$53</definedName>
     <definedName name="GAVI_countries">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="61">
   <si>
     <t>Measles</t>
   </si>
@@ -217,6 +217,18 @@
   </si>
   <si>
     <t>antigen demand</t>
+  </si>
+  <si>
+    <t>.025 demand</t>
+  </si>
+  <si>
+    <t>Rand</t>
+  </si>
+  <si>
+    <t>ran val</t>
+  </si>
+  <si>
+    <t>rand</t>
   </si>
 </sst>
 </file>
@@ -268,12 +280,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -299,7 +317,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -349,10 +367,9 @@
     <xf numFmtId="40" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -792,22 +809,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86710C76-81AC-48E5-8A5F-29B3CE6BD5DC}">
-  <dimension ref="A1:S52"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="8.85546875" style="2"/>
     <col min="5" max="5" width="16.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="18.42578125" customWidth="1"/>
-    <col min="18" max="18" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="18.42578125" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -823,9 +839,9 @@
       <c r="E1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -838,20 +854,18 @@
       <c r="D2" s="2">
         <v>2</v>
       </c>
-      <c r="E2" s="21">
-        <f>F2*2</f>
-        <v>8995469.8673202507</v>
-      </c>
-      <c r="F2" s="10">
-        <f>Medium_Capacity!J2*Medium_Capacity!K2</f>
-        <v>4497734.9336601254</v>
-      </c>
-      <c r="G2">
-        <f ca="1">RAND()</f>
-        <v>1.1167795206885933E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <f>ROUND(F2*G2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -864,20 +878,18 @@
       <c r="D3" s="2">
         <v>2</v>
       </c>
-      <c r="E3" s="21">
-        <f t="shared" ref="E3:E52" si="0">F3*2</f>
-        <v>1082008.0113759262</v>
-      </c>
-      <c r="F3" s="10">
-        <f>Medium_Capacity!J3*Medium_Capacity!K3</f>
-        <v>541004.0056879631</v>
-      </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G52" ca="1" si="1">RAND()</f>
-        <v>0.24372390434141256</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <f>ROUND(F3*G3,0)</f>
+        <v>26598928</v>
+      </c>
+      <c r="F3">
+        <v>13299464</v>
+      </c>
+      <c r="G3" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -890,20 +902,21 @@
       <c r="D4" s="2">
         <v>2</v>
       </c>
-      <c r="E4" s="21">
-        <f t="shared" si="0"/>
-        <v>201663047.818445</v>
-      </c>
-      <c r="F4" s="10">
-        <f>Medium_Capacity!J4*Medium_Capacity!K4</f>
-        <v>100831523.9092225</v>
-      </c>
-      <c r="G4">
-        <f ca="1">RAND()</f>
-        <v>0.16102113417165753</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <f t="shared" ref="E4:E52" si="0">ROUND(F4*G4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="22">
+        <v>2</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -916,20 +929,21 @@
       <c r="D5" s="2">
         <v>2</v>
       </c>
-      <c r="E5" s="21">
-        <f t="shared" si="0"/>
-        <v>33306249.520743433</v>
-      </c>
-      <c r="F5" s="10">
-        <f>Medium_Capacity!J5*Medium_Capacity!K5</f>
-        <v>16653124.760371717</v>
-      </c>
-      <c r="G5">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.38850828399846826</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E5" s="7">
+        <f>ROUND(F5*G5,0)</f>
+        <v>180558298</v>
+      </c>
+      <c r="F5">
+        <v>90279149</v>
+      </c>
+      <c r="G5" s="22">
+        <v>2</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -942,20 +956,21 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="21">
-        <f t="shared" si="0"/>
-        <v>15859003.458618619</v>
-      </c>
-      <c r="F6" s="10">
-        <f>Medium_Capacity!J6*Medium_Capacity!K6</f>
-        <v>7929501.7293093093</v>
-      </c>
-      <c r="G6">
-        <f t="shared" ca="1" si="1"/>
-        <v>2.1628095641952338E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>27094242</v>
+      </c>
+      <c r="F6">
+        <v>13547121</v>
+      </c>
+      <c r="G6" s="22">
+        <v>2</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -968,20 +983,21 @@
       <c r="D7" s="2">
         <v>2</v>
       </c>
-      <c r="E7" s="21">
-        <f t="shared" si="0"/>
-        <v>26934327.386733636</v>
-      </c>
-      <c r="F7" s="10">
-        <f>Medium_Capacity!J7*Medium_Capacity!K7</f>
-        <v>13467163.693366818</v>
-      </c>
-      <c r="G7">
-        <f ca="1">RAND()</f>
-        <v>0.4708381324509493</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>25010068</v>
+      </c>
+      <c r="F7">
+        <v>12505034</v>
+      </c>
+      <c r="G7" s="22">
+        <v>2</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -994,20 +1010,21 @@
       <c r="D8" s="2">
         <v>2</v>
       </c>
-      <c r="E8" s="21">
-        <f t="shared" si="0"/>
-        <v>50716.077929282517</v>
-      </c>
-      <c r="F8" s="10">
-        <f>Medium_Capacity!J8*Medium_Capacity!K8</f>
-        <v>25358.038964641259</v>
-      </c>
-      <c r="G8">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.84212910485942838</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>4364748</v>
+      </c>
+      <c r="F8">
+        <v>2182374</v>
+      </c>
+      <c r="G8" s="22">
+        <v>2</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -1020,20 +1037,21 @@
       <c r="D9" s="2">
         <v>2</v>
       </c>
-      <c r="E9" s="21">
-        <f t="shared" si="0"/>
-        <v>4370775.7851483794</v>
-      </c>
-      <c r="F9" s="10">
-        <f>Medium_Capacity!J9*Medium_Capacity!K9</f>
-        <v>2185387.8925741897</v>
-      </c>
-      <c r="G9">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.4584572715776597</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>8668850</v>
+      </c>
+      <c r="F9" s="23">
+        <v>4334425</v>
+      </c>
+      <c r="G9" s="22">
+        <v>2</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1046,20 +1064,21 @@
       <c r="D10" s="2">
         <v>2</v>
       </c>
-      <c r="E10" s="21">
-        <f t="shared" si="0"/>
-        <v>525732.89502522477</v>
-      </c>
-      <c r="F10" s="10">
-        <f>Medium_Capacity!J10*Medium_Capacity!K10</f>
-        <v>262866.44751261239</v>
-      </c>
-      <c r="G10">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.74861864536238298</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" s="22">
+        <v>2</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1072,20 +1091,18 @@
       <c r="D11" s="2">
         <v>2</v>
       </c>
-      <c r="E11" s="21">
-        <f t="shared" si="0"/>
-        <v>109565.26028398766</v>
-      </c>
-      <c r="F11" s="10">
-        <f>Medium_Capacity!J11*Medium_Capacity!K11</f>
-        <v>54782.630141993832</v>
-      </c>
-      <c r="G11">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.42714055396905537</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1098,20 +1115,18 @@
       <c r="D12" s="2">
         <v>2</v>
       </c>
-      <c r="E12" s="21">
-        <f t="shared" si="0"/>
-        <v>36221615.635631569</v>
-      </c>
-      <c r="F12" s="10">
-        <f>Medium_Capacity!J12*Medium_Capacity!K12</f>
-        <v>18110807.817815784</v>
-      </c>
-      <c r="G12">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.87703552032451393</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1124,20 +1139,18 @@
       <c r="D13" s="2">
         <v>2</v>
       </c>
-      <c r="E13" s="21">
-        <f t="shared" si="0"/>
-        <v>2264375.8518894236</v>
-      </c>
-      <c r="F13" s="10">
-        <f>Medium_Capacity!J13*Medium_Capacity!K13</f>
-        <v>1132187.9259447118</v>
-      </c>
-      <c r="G13">
-        <f ca="1">RAND()</f>
-        <v>0.7361746888080003</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -1150,20 +1163,18 @@
       <c r="D14" s="2">
         <v>2</v>
       </c>
-      <c r="E14" s="21">
-        <f t="shared" si="0"/>
-        <v>564690.75459061365</v>
-      </c>
-      <c r="F14" s="10">
-        <f>Medium_Capacity!J14*Medium_Capacity!K14</f>
-        <v>282345.37729530683</v>
-      </c>
-      <c r="G14">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.69764215936209439</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1176,20 +1187,18 @@
       <c r="D15" s="2">
         <v>2</v>
       </c>
-      <c r="E15" s="21">
-        <f t="shared" si="0"/>
-        <v>60932.701686140834</v>
-      </c>
-      <c r="F15" s="10">
-        <f>Medium_Capacity!J15*Medium_Capacity!K15</f>
-        <v>30466.350843070417</v>
-      </c>
-      <c r="G15">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.81273691459694963</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -1202,20 +1211,21 @@
       <c r="D16" s="2">
         <v>2</v>
       </c>
-      <c r="E16" s="21">
-        <f t="shared" si="0"/>
-        <v>17.475918265623562</v>
-      </c>
-      <c r="F16" s="10">
-        <f>Medium_Capacity!J16*Medium_Capacity!K16</f>
-        <v>8.7379591328117812</v>
-      </c>
-      <c r="G16">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.905814016649933</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F16" s="23">
+        <v>0</v>
+      </c>
+      <c r="G16" s="22">
+        <v>2</v>
+      </c>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1228,20 +1238,19 @@
       <c r="D17" s="2">
         <v>2</v>
       </c>
-      <c r="E17" s="21">
-        <f t="shared" si="0"/>
-        <v>3188220.3996289601</v>
-      </c>
-      <c r="F17" s="10">
-        <f>Medium_Capacity!J17*Medium_Capacity!K17</f>
-        <v>1594110.19981448</v>
-      </c>
-      <c r="G17">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.34991316527751914</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>80427884</v>
+      </c>
+      <c r="F17">
+        <v>40213942</v>
+      </c>
+      <c r="G17" s="22">
+        <v>2</v>
+      </c>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1254,20 +1263,19 @@
       <c r="D18" s="2">
         <v>2</v>
       </c>
-      <c r="E18" s="21">
-        <f t="shared" si="0"/>
-        <v>662897.31081394223</v>
-      </c>
-      <c r="F18" s="10">
-        <f>Medium_Capacity!J18*Medium_Capacity!K18</f>
-        <v>331448.65540697111</v>
-      </c>
-      <c r="G18">
-        <f ca="1">RAND()</f>
-        <v>0.97803305077510982</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" s="22">
+        <v>2</v>
+      </c>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1280,20 +1288,19 @@
       <c r="D19" s="2">
         <v>2</v>
       </c>
-      <c r="E19" s="21">
-        <f t="shared" si="0"/>
-        <v>441931.54054262809</v>
-      </c>
-      <c r="F19" s="10">
-        <f>Medium_Capacity!J19*Medium_Capacity!K19</f>
-        <v>220965.77027131405</v>
-      </c>
-      <c r="G19">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.1746677472978041</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" s="22">
+        <v>2</v>
+      </c>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1306,20 +1313,19 @@
       <c r="D20" s="2">
         <v>2</v>
       </c>
-      <c r="E20" s="21">
-        <f t="shared" si="0"/>
-        <v>5503099.8977093929</v>
-      </c>
-      <c r="F20" s="10">
-        <f>Medium_Capacity!J20*Medium_Capacity!K20</f>
-        <v>2751549.9488546965</v>
-      </c>
-      <c r="G20">
-        <f t="shared" ca="1" si="1"/>
-        <v>8.9593362192195714E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>86730208</v>
+      </c>
+      <c r="F20">
+        <v>43365104</v>
+      </c>
+      <c r="G20" s="22">
+        <v>2</v>
+      </c>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1332,20 +1338,18 @@
       <c r="D21" s="2">
         <v>2</v>
       </c>
-      <c r="E21" s="21">
-        <f t="shared" si="0"/>
-        <v>266873655.20470208</v>
-      </c>
-      <c r="F21" s="10">
-        <f>Medium_Capacity!J21*Medium_Capacity!K21</f>
-        <v>133436827.60235104</v>
-      </c>
-      <c r="G21">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.60865941991703798</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1358,21 +1362,19 @@
       <c r="D22" s="2">
         <v>2</v>
       </c>
-      <c r="E22" s="21">
-        <f t="shared" si="0"/>
-        <v>32100539.184251159</v>
-      </c>
-      <c r="F22" s="10">
-        <f>Medium_Capacity!J22*Medium_Capacity!K22</f>
-        <v>16050269.59212558</v>
-      </c>
-      <c r="G22">
-        <f t="shared" ca="1" si="1"/>
-        <v>4.3346483646909073E-2</v>
-      </c>
-      <c r="R22" s="10"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>84680592</v>
+      </c>
+      <c r="F22">
+        <v>42340296</v>
+      </c>
+      <c r="G22" s="22">
+        <v>2</v>
+      </c>
+      <c r="O22" s="10"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -1385,21 +1387,19 @@
       <c r="D23" s="2">
         <v>2</v>
       </c>
-      <c r="E23" s="21">
-        <f t="shared" si="0"/>
-        <v>453248050.48020494</v>
-      </c>
-      <c r="F23" s="10">
-        <f>Medium_Capacity!J23*Medium_Capacity!K23</f>
-        <v>226624025.24010247</v>
-      </c>
-      <c r="G23">
-        <f t="shared" ca="1" si="1"/>
-        <v>7.7260058632008355E-2</v>
-      </c>
-      <c r="R23" s="10"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>438402962</v>
+      </c>
+      <c r="F23">
+        <v>219201481</v>
+      </c>
+      <c r="G23" s="22">
+        <v>2</v>
+      </c>
+      <c r="O23" s="10"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -1412,21 +1412,20 @@
       <c r="D24" s="2">
         <v>2</v>
       </c>
-      <c r="E24" s="21">
-        <f t="shared" si="0"/>
-        <v>28796881.635271627</v>
-      </c>
-      <c r="F24" s="10">
-        <f>Medium_Capacity!J24*Medium_Capacity!K24</f>
-        <v>14398440.817635814</v>
-      </c>
-      <c r="G24">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.33742665490780799</v>
-      </c>
-      <c r="R24" s="10"/>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E24">
+        <f t="shared" si="0"/>
+        <v>122441776</v>
+      </c>
+      <c r="F24">
+        <v>61220888</v>
+      </c>
+      <c r="G24" s="22">
+        <v>2</v>
+      </c>
+      <c r="J24" s="2"/>
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -1439,21 +1438,20 @@
       <c r="D25" s="2">
         <v>2</v>
       </c>
-      <c r="E25" s="21">
-        <f t="shared" si="0"/>
-        <v>5643748.3128400408</v>
-      </c>
-      <c r="F25" s="10">
-        <f>Medium_Capacity!J25*Medium_Capacity!K25</f>
-        <v>2821874.1564200204</v>
-      </c>
-      <c r="G25">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.61522145884882029</v>
-      </c>
-      <c r="R25" s="10"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" s="22">
+        <v>2</v>
+      </c>
+      <c r="J25" s="2"/>
+      <c r="O25" s="10"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -1466,21 +1464,21 @@
       <c r="D26" s="2">
         <v>2</v>
       </c>
-      <c r="E26" s="21">
-        <f t="shared" si="0"/>
-        <v>2202438.3659863574</v>
-      </c>
-      <c r="F26" s="10">
-        <f>Medium_Capacity!J26*Medium_Capacity!K26</f>
-        <v>1101219.1829931787</v>
-      </c>
-      <c r="G26">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.7542202566351679</v>
-      </c>
-      <c r="R26" s="10"/>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="22">
+        <v>2</v>
+      </c>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="O26" s="10"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -1493,21 +1491,21 @@
       <c r="D27" s="2">
         <v>2</v>
       </c>
-      <c r="E27" s="21">
-        <f t="shared" si="0"/>
-        <v>9910972.646938609</v>
-      </c>
-      <c r="F27" s="10">
-        <f>Medium_Capacity!J27*Medium_Capacity!K27</f>
-        <v>4955486.3234693045</v>
-      </c>
-      <c r="G27">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.78888100396314265</v>
-      </c>
-      <c r="R27" s="10"/>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" s="22">
+        <v>2</v>
+      </c>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="O27" s="10"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -1520,21 +1518,21 @@
       <c r="D28" s="2">
         <v>2</v>
       </c>
-      <c r="E28" s="21">
-        <f t="shared" si="0"/>
-        <v>2202438.3659863574</v>
-      </c>
-      <c r="F28" s="10">
-        <f>Medium_Capacity!J28*Medium_Capacity!K28</f>
-        <v>1101219.1829931787</v>
-      </c>
-      <c r="G28">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.6563546955005799</v>
-      </c>
-      <c r="R28" s="10"/>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E28">
+        <f t="shared" si="0"/>
+        <v>12000000</v>
+      </c>
+      <c r="F28" s="23">
+        <v>6000000</v>
+      </c>
+      <c r="G28" s="22">
+        <v>2</v>
+      </c>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="O28" s="10"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>41</v>
       </c>
@@ -1547,21 +1545,20 @@
       <c r="D29" s="2">
         <v>2</v>
       </c>
-      <c r="E29" s="21">
-        <f t="shared" si="0"/>
-        <v>3898923.4682316827</v>
-      </c>
-      <c r="F29" s="10">
-        <f>Medium_Capacity!J29*Medium_Capacity!K29</f>
-        <v>1949461.7341158413</v>
-      </c>
-      <c r="G29">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.38840384713949938</v>
-      </c>
-      <c r="R29" s="10"/>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" s="22">
+        <v>2</v>
+      </c>
+      <c r="J29" s="2"/>
+      <c r="O29" s="10"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -1574,20 +1571,18 @@
       <c r="D30" s="2">
         <v>2</v>
       </c>
-      <c r="E30" s="21">
-        <f t="shared" si="0"/>
-        <v>468976.77281920932</v>
-      </c>
-      <c r="F30" s="10">
-        <f>Medium_Capacity!J30*Medium_Capacity!K30</f>
-        <v>234488.38640960466</v>
-      </c>
-      <c r="G30">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.97464368473240415</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E30">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -1600,24 +1595,22 @@
       <c r="D31" s="2">
         <v>2</v>
       </c>
-      <c r="E31" s="21">
-        <f t="shared" si="0"/>
-        <v>97737.011831104493</v>
-      </c>
-      <c r="F31" s="10">
-        <f>Medium_Capacity!J31*Medium_Capacity!K31</f>
-        <v>48868.505915552247</v>
-      </c>
-      <c r="G31">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.31683031621759328</v>
-      </c>
-      <c r="R31" s="18"/>
-      <c r="S31" t="s">
+      <c r="E31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31" s="22">
+        <v>2</v>
+      </c>
+      <c r="O31" s="18"/>
+      <c r="P31" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -1630,20 +1623,18 @@
       <c r="D32" s="2">
         <v>2</v>
       </c>
-      <c r="E32" s="21">
-        <f t="shared" si="0"/>
-        <v>148217673.40024289</v>
-      </c>
-      <c r="F32" s="10">
-        <f>Medium_Capacity!J32*Medium_Capacity!K32</f>
-        <v>74108836.700121447</v>
-      </c>
-      <c r="G32">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.89544319310233889</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>360354112</v>
+      </c>
+      <c r="F32">
+        <v>180177056</v>
+      </c>
+      <c r="G32" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -1656,20 +1647,18 @@
       <c r="D33" s="2">
         <v>2</v>
       </c>
-      <c r="E33" s="21">
-        <f t="shared" si="0"/>
-        <v>17828163.777101099</v>
-      </c>
-      <c r="F33" s="10">
-        <f>Medium_Capacity!J33*Medium_Capacity!K33</f>
-        <v>8914081.8885505497</v>
-      </c>
-      <c r="G33">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.80324100620154315</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E33">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1682,20 +1671,18 @@
       <c r="D34" s="2">
         <v>2</v>
       </c>
-      <c r="E34" s="21">
-        <f t="shared" si="0"/>
-        <v>3715474.955262064</v>
-      </c>
-      <c r="F34" s="10">
-        <f>Medium_Capacity!J34*Medium_Capacity!K34</f>
-        <v>1857737.477631032</v>
-      </c>
-      <c r="G34">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.98922134145888607</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E34">
+        <f t="shared" si="0"/>
+        <v>26610904</v>
+      </c>
+      <c r="F34">
+        <v>13305452</v>
+      </c>
+      <c r="G34" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1708,20 +1695,19 @@
       <c r="D35" s="2">
         <v>2</v>
       </c>
-      <c r="E35" s="21">
-        <f t="shared" si="0"/>
-        <v>37774877.613046914</v>
-      </c>
-      <c r="F35" s="10">
-        <f>Medium_Capacity!J35*Medium_Capacity!K35</f>
-        <v>18887438.806523457</v>
-      </c>
-      <c r="G35">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.52809839143432613</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E35">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35" s="22">
+        <v>2</v>
+      </c>
+      <c r="J35" s="2"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1734,20 +1720,19 @@
       <c r="D36" s="2">
         <v>2</v>
       </c>
-      <c r="E36" s="21">
-        <f t="shared" si="0"/>
-        <v>6238820.2152353404</v>
-      </c>
-      <c r="F36" s="10">
-        <f>Medium_Capacity!J36*Medium_Capacity!K36</f>
-        <v>3119410.1076176702</v>
-      </c>
-      <c r="G36">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.40794493376031726</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E36">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36" s="22">
+        <v>2</v>
+      </c>
+      <c r="J36" s="2"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1760,20 +1745,19 @@
       <c r="D37" s="2">
         <v>2</v>
       </c>
-      <c r="E37" s="21">
-        <f t="shared" si="0"/>
-        <v>3546873.5784291485</v>
-      </c>
-      <c r="F37" s="10">
-        <f>Medium_Capacity!J37*Medium_Capacity!K37</f>
-        <v>1773436.7892145743</v>
-      </c>
-      <c r="G37">
-        <f t="shared" ca="1" si="1"/>
-        <v>7.1825410299488301E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37" s="22">
+        <v>2</v>
+      </c>
+      <c r="J37" s="2"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>29</v>
       </c>
@@ -1786,20 +1770,18 @@
       <c r="D38" s="2">
         <v>2</v>
       </c>
-      <c r="E38" s="21">
-        <f t="shared" si="0"/>
-        <v>153878658.90735054</v>
-      </c>
-      <c r="F38" s="10">
-        <f>Medium_Capacity!J38*Medium_Capacity!K38</f>
-        <v>76939329.45367527</v>
-      </c>
-      <c r="G38">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.7019548579452014</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E38">
+        <f t="shared" si="0"/>
+        <v>281863128</v>
+      </c>
+      <c r="F38">
+        <v>140931564</v>
+      </c>
+      <c r="G38" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>29</v>
       </c>
@@ -1812,20 +1794,18 @@
       <c r="D39" s="2">
         <v>2</v>
       </c>
-      <c r="E39" s="21">
-        <f t="shared" si="0"/>
-        <v>18509087.815680332</v>
-      </c>
-      <c r="F39" s="10">
-        <f>Medium_Capacity!J39*Medium_Capacity!K39</f>
-        <v>9254543.9078401662</v>
-      </c>
-      <c r="G39">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.29860537905155371</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E39">
+        <f t="shared" si="0"/>
+        <v>62636250</v>
+      </c>
+      <c r="F39">
+        <v>31318125</v>
+      </c>
+      <c r="G39" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -1838,20 +1818,18 @@
       <c r="D40" s="2">
         <v>2</v>
       </c>
-      <c r="E40" s="21">
-        <f t="shared" si="0"/>
-        <v>25414279.239197437</v>
-      </c>
-      <c r="F40" s="10">
-        <f>Medium_Capacity!J40*Medium_Capacity!K40</f>
-        <v>12707139.619598718</v>
-      </c>
-      <c r="G40">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.4319270722200973</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E40" s="7">
+        <f t="shared" si="0"/>
+        <v>107376430</v>
+      </c>
+      <c r="F40">
+        <v>53688215</v>
+      </c>
+      <c r="G40" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>29</v>
       </c>
@@ -1864,20 +1842,18 @@
       <c r="D41" s="2">
         <v>2</v>
       </c>
-      <c r="E41" s="21">
-        <f t="shared" si="0"/>
-        <v>9619645.9831065871</v>
-      </c>
-      <c r="F41" s="10">
-        <f>Medium_Capacity!J41*Medium_Capacity!K41</f>
-        <v>4809822.9915532935</v>
-      </c>
-      <c r="G41">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.61363707064142503</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E41">
+        <f t="shared" si="0"/>
+        <v>35792142</v>
+      </c>
+      <c r="F41">
+        <v>17896071</v>
+      </c>
+      <c r="G41" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>29</v>
       </c>
@@ -1890,20 +1866,18 @@
       <c r="D42" s="2">
         <v>2</v>
       </c>
-      <c r="E42" s="21">
-        <f t="shared" si="0"/>
-        <v>3254170.6708528879</v>
-      </c>
-      <c r="F42" s="10">
-        <f>Medium_Capacity!J42*Medium_Capacity!K42</f>
-        <v>1627085.335426444</v>
-      </c>
-      <c r="G42">
-        <f t="shared" ca="1" si="1"/>
-        <v>9.5270347599945793E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E42">
+        <f t="shared" si="0"/>
+        <v>17896070</v>
+      </c>
+      <c r="F42">
+        <v>8948035</v>
+      </c>
+      <c r="G42" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -1916,20 +1890,18 @@
       <c r="D43" s="2">
         <v>2</v>
       </c>
-      <c r="E43" s="21">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F43" s="10">
-        <f>Medium_Capacity!J43*Medium_Capacity!K43</f>
-        <v>0</v>
-      </c>
-      <c r="G43">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.16522897829660532</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>9</v>
       </c>
@@ -1942,20 +1914,18 @@
       <c r="D44" s="2">
         <v>2</v>
       </c>
-      <c r="E44" s="21">
-        <f t="shared" si="0"/>
-        <v>19631183.599143814</v>
-      </c>
-      <c r="F44" s="10">
-        <f>Medium_Capacity!J44*Medium_Capacity!K44</f>
-        <v>9815591.7995719071</v>
-      </c>
-      <c r="G44">
-        <f t="shared" ca="1" si="1"/>
-        <v>4.4050972493482776E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E44">
+        <f t="shared" si="0"/>
+        <v>26928732</v>
+      </c>
+      <c r="F44">
+        <v>13464366</v>
+      </c>
+      <c r="G44" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -1968,20 +1938,18 @@
       <c r="D45" s="2">
         <v>2</v>
       </c>
-      <c r="E45" s="21">
-        <f t="shared" si="0"/>
-        <v>36964.599968017625</v>
-      </c>
-      <c r="F45" s="10">
-        <f>Medium_Capacity!J45*Medium_Capacity!K45</f>
-        <v>18482.299984008812</v>
-      </c>
-      <c r="G45">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.1426593193032869</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E45">
+        <f t="shared" si="0"/>
+        <v>1450008</v>
+      </c>
+      <c r="F45">
+        <v>725004</v>
+      </c>
+      <c r="G45" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>9</v>
       </c>
@@ -1994,20 +1962,18 @@
       <c r="D46" s="2">
         <v>2</v>
       </c>
-      <c r="E46" s="21">
-        <f t="shared" si="0"/>
-        <v>5962.0322529060686</v>
-      </c>
-      <c r="F46" s="10">
-        <f>Medium_Capacity!J46*Medium_Capacity!K46</f>
-        <v>2981.0161264530343</v>
-      </c>
-      <c r="G46">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.20292478695050098</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>10</v>
       </c>
@@ -2020,20 +1986,18 @@
       <c r="D47" s="2">
         <v>2</v>
       </c>
-      <c r="E47" s="21">
-        <f t="shared" si="0"/>
-        <v>86732745.238201126</v>
-      </c>
-      <c r="F47" s="10">
-        <f>Medium_Capacity!J47*Medium_Capacity!K47</f>
-        <v>43366372.619100563</v>
-      </c>
-      <c r="G47">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.61864953883212725</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47" s="22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>10</v>
       </c>
@@ -2046,17 +2010,15 @@
       <c r="D48" s="2">
         <v>2</v>
       </c>
-      <c r="E48" s="21">
-        <f t="shared" si="0"/>
-        <v>147303590.76416737</v>
-      </c>
-      <c r="F48" s="10">
-        <f>Medium_Capacity!J48*Medium_Capacity!K48</f>
-        <v>73651795.382083684</v>
-      </c>
-      <c r="G48">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.79522251913334219</v>
+      <c r="E48">
+        <f t="shared" si="0"/>
+        <v>113020800</v>
+      </c>
+      <c r="F48">
+        <v>56510400</v>
+      </c>
+      <c r="G48" s="22">
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -2072,17 +2034,15 @@
       <c r="D49" s="2">
         <v>2</v>
       </c>
-      <c r="E49" s="21">
-        <f t="shared" si="0"/>
-        <v>3221021.8164485223</v>
-      </c>
-      <c r="F49" s="10">
-        <f>Medium_Capacity!J49*Medium_Capacity!K49</f>
-        <v>1610510.9082242611</v>
-      </c>
-      <c r="G49">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.52439698246154198</v>
+      <c r="E49">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49" s="22">
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -2098,17 +2058,15 @@
       <c r="D50" s="2">
         <v>2</v>
       </c>
-      <c r="E50" s="21">
-        <f t="shared" si="0"/>
-        <v>97885620.44911465</v>
-      </c>
-      <c r="F50" s="10">
-        <f>Medium_Capacity!J50*Medium_Capacity!K50</f>
-        <v>48942810.224557325</v>
-      </c>
-      <c r="G50">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.12963608598244625</v>
+      <c r="E50">
+        <f t="shared" si="0"/>
+        <v>297066666</v>
+      </c>
+      <c r="F50">
+        <v>148533333</v>
+      </c>
+      <c r="G50" s="22">
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -2124,17 +2082,15 @@
       <c r="D51" s="2">
         <v>2</v>
       </c>
-      <c r="E51" s="21">
-        <f t="shared" si="0"/>
-        <v>166245209.19674805</v>
-      </c>
-      <c r="F51" s="10">
-        <f>Medium_Capacity!J51*Medium_Capacity!K51</f>
-        <v>83122604.598374024</v>
-      </c>
-      <c r="G51">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.84642157663473161</v>
+      <c r="E51">
+        <f t="shared" si="0"/>
+        <v>371326084</v>
+      </c>
+      <c r="F51">
+        <v>185663042</v>
+      </c>
+      <c r="G51" s="22">
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -2150,21 +2106,19 @@
       <c r="D52" s="2">
         <v>2</v>
       </c>
-      <c r="E52" s="21">
-        <f t="shared" si="0"/>
-        <v>585672.67794888001</v>
-      </c>
-      <c r="F52" s="10">
-        <f>Medium_Capacity!J52*Medium_Capacity!K52</f>
-        <v>292836.33897444</v>
-      </c>
-      <c r="G52">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.79328300225326998</v>
+      <c r="E52">
+        <f t="shared" si="0"/>
+        <v>8000000</v>
+      </c>
+      <c r="F52">
+        <v>4000000</v>
+      </c>
+      <c r="G52" s="22">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S53" xr:uid="{86710C76-81AC-48E5-8A5F-29B3CE6BD5DC}"/>
+  <autoFilter ref="A1:P53" xr:uid="{86710C76-81AC-48E5-8A5F-29B3CE6BD5DC}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2172,138 +2126,220 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFBA2FAA-95C5-423D-A8C0-3A912D67D407}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
       <c r="B1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
       <c r="B2">
-        <f>C2</f>
-        <v>3694295.5570033002</v>
+        <f>ROUND(C2,0)</f>
+        <v>3694296</v>
       </c>
       <c r="C2">
         <f>Medium_Capacity!C49*0.25</f>
         <v>3694295.5570033002</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <f ca="1">RAND()</f>
+        <v>0.67428318662036768</v>
+      </c>
+      <c r="E2">
+        <f ca="1">C2*D2</f>
+        <v>2491001.3804936516</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B18" si="0">C3</f>
-        <v>82819787.354738995</v>
+        <f t="shared" ref="B3:B18" si="0">ROUND(C3,0)</f>
+        <v>82819787</v>
       </c>
       <c r="C3">
         <f>Medium_Capacity!C50*0.25</f>
         <v>82819787.354738995</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <f t="shared" ref="D3:D18" ca="1" si="1">RAND()</f>
+        <v>1.9195167969764837E-2</v>
+      </c>
+      <c r="E3">
+        <f ca="1">C3*D3</f>
+        <v>1589739.7294944208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
-        <v>6513038.9940517964</v>
+        <v>6513039</v>
       </c>
       <c r="C4">
         <f>Medium_Capacity!C51*0.25</f>
         <v>6513038.9940517964</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.37522173218852128</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E18" ca="1" si="2">C4*D4</f>
+        <v>2443833.7731594993</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
       <c r="B5">
         <f t="shared" si="0"/>
-        <v>1795007.6874129353</v>
+        <v>1795008</v>
       </c>
       <c r="C5">
         <f>Medium_Capacity!C52*0.25</f>
         <v>1795007.6874129353</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.65546107918652752</v>
+      </c>
+      <c r="E5">
+        <f ca="1">C5*D5</f>
+        <v>1176557.6759397956</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
       <c r="B6">
         <f t="shared" si="0"/>
-        <v>60870627.147684671</v>
+        <v>60870627</v>
       </c>
       <c r="C6">
         <f>Medium_Capacity!C53*0.25</f>
         <v>60870627.147684671</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.15565862294510568</v>
+      </c>
+      <c r="E6">
+        <f ca="1">C6*D6</f>
+        <v>9475037.9996135626</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
       <c r="B7">
         <f t="shared" si="0"/>
-        <v>1601225.4899671054</v>
+        <v>1601225</v>
       </c>
       <c r="C7">
         <f>Medium_Capacity!C54*0.25</f>
         <v>1601225.4899671054</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.97557197921062289</v>
+      </c>
+      <c r="E7">
+        <f ca="1">C7*D7</f>
+        <v>1562110.7204097083</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>42</v>
       </c>
       <c r="B8">
         <f t="shared" si="0"/>
-        <v>15513537.879683325</v>
+        <v>15513538</v>
       </c>
       <c r="C8">
         <f>Medium_Capacity!C55*0.25</f>
         <v>15513537.879683325</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.64565072216885733</v>
+      </c>
+      <c r="E8">
+        <f t="shared" ca="1" si="2"/>
+        <v>10016326.935411463</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
       <c r="B9">
         <f t="shared" si="0"/>
-        <v>1456644.232631579</v>
+        <v>1456644</v>
       </c>
       <c r="C9">
         <f>Medium_Capacity!C56*0.25</f>
         <v>1456644.232631579</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.33294300625874085</v>
+      </c>
+      <c r="E9">
+        <f t="shared" ca="1" si="2"/>
+        <v>484979.50986181456</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
       <c r="B10">
         <f t="shared" si="0"/>
-        <v>63195503.325986847</v>
+        <v>63195503</v>
       </c>
       <c r="C10">
         <f>Medium_Capacity!C57*0.25</f>
         <v>63195503.325986847</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.25262624793587207</v>
+      </c>
+      <c r="E10">
+        <f t="shared" ca="1" si="2"/>
+        <v>15964842.891662981</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -2315,96 +2351,160 @@
         <f>Medium_Capacity!C58*0.25</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.70299570777977005</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
       <c r="B12">
         <f t="shared" si="0"/>
-        <v>20944761.71187168</v>
+        <v>20944762</v>
       </c>
       <c r="C12">
         <f>Medium_Capacity!C59*0.25</f>
         <v>20944761.71187168</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.98782305486119371</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ca="1" si="2"/>
+        <v>20689718.497560848</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>34</v>
       </c>
       <c r="B13">
         <f t="shared" si="0"/>
-        <v>109600740.51114175</v>
+        <v>109600741</v>
       </c>
       <c r="C13">
         <f>Medium_Capacity!C60*0.25</f>
         <v>109600740.51114175</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.55447524006993898</v>
+      </c>
+      <c r="E13">
+        <f t="shared" ca="1" si="2"/>
+        <v>60770896.906758405</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
       <c r="B14">
         <f t="shared" si="0"/>
-        <v>4747052.4303343054</v>
+        <v>4747052</v>
       </c>
       <c r="C14">
         <f>Medium_Capacity!C61*0.25</f>
         <v>4747052.4303343054</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.18756321685715038</v>
+      </c>
+      <c r="E14">
+        <f t="shared" ca="1" si="2"/>
+        <v>890372.42442305607</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
       <c r="B15">
         <f t="shared" si="0"/>
-        <v>14875638.036021562</v>
+        <v>14875638</v>
       </c>
       <c r="C15">
         <f>Medium_Capacity!C62*0.25</f>
         <v>14875638.036021562</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.95265802543902234</v>
+      </c>
+      <c r="E15">
+        <f t="shared" ca="1" si="2"/>
+        <v>14171395.958541919</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
       <c r="B16">
         <f t="shared" si="0"/>
-        <v>231909.45848684211</v>
+        <v>231909</v>
       </c>
       <c r="C16">
         <f>Medium_Capacity!C63*0.25</f>
-        <v>231909.45848684211</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>231909.45848684199</v>
+      </c>
+      <c r="D16">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.94695191832779779</v>
+      </c>
+      <c r="E16">
+        <f t="shared" ca="1" si="2"/>
+        <v>219607.10659247581</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
       <c r="B17">
         <f t="shared" si="0"/>
-        <v>35619750.841946572</v>
+        <v>35619751</v>
       </c>
       <c r="C17">
         <f>Medium_Capacity!C64*0.25</f>
         <v>35619750.841946572</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.61844424334864745</v>
+      </c>
+      <c r="E17">
+        <f t="shared" ca="1" si="2"/>
+        <v>22028829.857714996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18">
         <f t="shared" si="0"/>
-        <v>40200058.257479519</v>
+        <v>40200058</v>
       </c>
       <c r="C18">
         <f>Medium_Capacity!C65*0.25</f>
         <v>40200058.257479519</v>
+      </c>
+      <c r="D18">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.52447587557571329</v>
+      </c>
+      <c r="E18">
+        <f t="shared" ca="1" si="2"/>
+        <v>21083960.752786253</v>
       </c>
     </row>
   </sheetData>
@@ -2414,163 +2514,215 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5C2B8D5-A351-43B6-AB72-03AAE787B34B}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="21">
         <f>C2</f>
         <v>37210000</v>
       </c>
       <c r="C2" s="19">
         <v>37210000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <f ca="1">RAND()</f>
+        <v>0.12224538017765141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="21">
         <f t="shared" ref="B3:B13" si="0">C3</f>
         <v>2610000</v>
       </c>
       <c r="C3" s="19">
         <v>2610000</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <f t="shared" ref="D3:D13" ca="1" si="1">RAND()</f>
+        <v>0.85421549097131677</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="21">
         <f t="shared" si="0"/>
         <v>35730000</v>
       </c>
       <c r="C4" s="19">
         <v>35730000</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.39993762364780461</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="21">
         <f t="shared" si="0"/>
         <v>5706000</v>
       </c>
       <c r="C5" s="19">
         <v>5706000</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.91022935118489534</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="21">
         <f t="shared" si="0"/>
         <v>5777000</v>
       </c>
       <c r="C6" s="19">
         <v>5777000</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.5779474952648499</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="21">
         <f t="shared" si="0"/>
         <v>3207000</v>
       </c>
       <c r="C7" s="19">
         <v>3207000</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.73205605409293717</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="21">
         <f t="shared" si="0"/>
         <v>2595000</v>
       </c>
       <c r="C8" s="19">
         <v>2595000</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.61790400483780106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="21">
         <f t="shared" si="0"/>
         <v>3123000</v>
       </c>
       <c r="C9" s="19">
         <v>3123000</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.22826908380477895</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="21">
         <f t="shared" si="0"/>
         <v>5222000</v>
       </c>
       <c r="C10" s="19">
         <v>5222000</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.36289577208311463</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="21">
         <f t="shared" si="0"/>
         <v>1900000</v>
       </c>
       <c r="C11" s="19">
         <v>1900000</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.25394492013263936</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="21">
         <f t="shared" si="0"/>
         <v>14250000</v>
       </c>
       <c r="C12" s="19">
         <v>14250000</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.96948719859735211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="21">
         <f t="shared" si="0"/>
         <v>1608000</v>
       </c>
       <c r="C13" s="19">
         <v>1608000</v>
+      </c>
+      <c r="D13">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.4956765337998843</v>
       </c>
     </row>
   </sheetData>
@@ -2586,7 +2738,7 @@
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.140625" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" customWidth="1"/>
@@ -2674,7 +2826,7 @@
         <v>46</v>
       </c>
       <c r="B2" s="8">
-        <v>25200000</v>
+        <v>12600000</v>
       </c>
       <c r="C2" s="17">
         <f>B2/$B$20</f>
@@ -2682,15 +2834,15 @@
       </c>
       <c r="D2" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A2)</f>
-        <v>662897.31081394223</v>
+        <v>0</v>
       </c>
       <c r="E2" s="15">
         <f>VLOOKUP(Medium_Capacity!A2, Medium_Capacity!A1:A18:B1:B18, 2, FALSE)</f>
-        <v>25200000</v>
+        <v>12600000</v>
       </c>
       <c r="F2" s="20">
         <f>E2-D2</f>
-        <v>24537102.689186059</v>
+        <v>12600000</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -2703,8 +2855,12 @@
         <f>VLOOKUP(Q_start!A2,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>14777182.228013201</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
+      <c r="L2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
@@ -2750,7 +2906,7 @@
         <v>28</v>
       </c>
       <c r="B3" s="8">
-        <v>48600000</v>
+        <v>24300000</v>
       </c>
       <c r="C3" s="17">
         <f t="shared" ref="C3:C18" si="0">B3/$B$20</f>
@@ -2758,15 +2914,15 @@
       </c>
       <c r="D3" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A3)</f>
-        <v>3922777.2273771563</v>
+        <v>26610904</v>
       </c>
       <c r="E3" s="15">
         <f>VLOOKUP(Medium_Capacity!A3, Medium_Capacity!A2:A19:B2:B19, 2, FALSE)</f>
-        <v>48600000</v>
+        <v>24300000</v>
       </c>
       <c r="F3" s="20">
-        <f t="shared" ref="F3:F7" si="1">E3-D3</f>
-        <v>44677222.772622846</v>
+        <f t="shared" ref="F3:F18" si="1">E3-D3</f>
+        <v>-2310904</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
@@ -2779,8 +2935,12 @@
         <f>VLOOKUP(Q_start!A3,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>14777182.228013201</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
+      <c r="L3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
@@ -2826,7 +2986,7 @@
         <v>48</v>
       </c>
       <c r="B4" s="8">
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="C4" s="17">
         <f t="shared" si="0"/>
@@ -2834,15 +2994,15 @@
       </c>
       <c r="D4" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A4)</f>
-        <v>2202438.3659863574</v>
+        <v>0</v>
       </c>
       <c r="E4" s="15">
         <f>VLOOKUP(Medium_Capacity!A4, Medium_Capacity!A3:A20:B3:B20, 2, FALSE)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="F4" s="20">
         <f t="shared" si="1"/>
-        <v>13797561.634013642</v>
+        <v>8000000</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
@@ -2855,8 +3015,12 @@
         <f>VLOOKUP(Q_start!A4,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>331279149.41895598</v>
       </c>
-      <c r="L4" s="6"/>
-      <c r="M4" s="5"/>
+      <c r="L4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
@@ -2902,23 +3066,23 @@
         <v>36</v>
       </c>
       <c r="B5" s="8">
-        <v>72000000</v>
+        <v>36000000</v>
       </c>
       <c r="C5" s="17">
-        <f t="shared" si="0"/>
+        <f>B5/$B$20</f>
         <v>1.1303496446188567E-2</v>
       </c>
       <c r="D5" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A5)</f>
-        <v>13131994.463387132</v>
+        <v>0</v>
       </c>
       <c r="E5" s="15">
         <f>VLOOKUP(Medium_Capacity!A5, Medium_Capacity!A4:A21:B4:B21, 2, FALSE)</f>
-        <v>72000000</v>
+        <v>36000000</v>
       </c>
       <c r="F5" s="20">
         <f t="shared" si="1"/>
-        <v>58868005.536612868</v>
+        <v>36000000</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -2931,8 +3095,12 @@
         <f>VLOOKUP(Q_start!A5,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>331279149.41895598</v>
       </c>
-      <c r="L5" s="6"/>
-      <c r="M5" s="5"/>
+      <c r="L5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
@@ -2978,7 +3146,7 @@
         <v>47</v>
       </c>
       <c r="B6" s="8">
-        <v>16800000</v>
+        <v>8400000</v>
       </c>
       <c r="C6" s="17">
         <f t="shared" si="0"/>
@@ -2986,15 +3154,15 @@
       </c>
       <c r="D6" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A6)</f>
-        <v>441931.54054262809</v>
+        <v>0</v>
       </c>
       <c r="E6" s="15">
         <f>VLOOKUP(Medium_Capacity!A6, Medium_Capacity!A5:A22:B5:B22, 2, FALSE)</f>
-        <v>16800000</v>
+        <v>8400000</v>
       </c>
       <c r="F6" s="20">
         <f t="shared" si="1"/>
-        <v>16358068.459457371</v>
+        <v>8400000</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -3007,8 +3175,12 @@
         <f>VLOOKUP(Q_start!A6,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>26052155.976207186</v>
       </c>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="L6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
@@ -3054,7 +3226,7 @@
         <v>26</v>
       </c>
       <c r="B7" s="8">
-        <v>320200000</v>
+        <v>160100000</v>
       </c>
       <c r="C7" s="17">
         <f t="shared" si="0"/>
@@ -3062,15 +3234,15 @@
       </c>
       <c r="D7" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A7)</f>
-        <v>64959348.975176215</v>
+        <v>287934728</v>
       </c>
       <c r="E7" s="15">
         <f>VLOOKUP(Medium_Capacity!A7, Medium_Capacity!A6:A23:B6:B23, 2, FALSE)</f>
-        <v>320200000</v>
+        <v>160100000</v>
       </c>
       <c r="F7" s="20">
         <f t="shared" si="1"/>
-        <v>255240651.02482378</v>
+        <v>-127834728</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -3083,8 +3255,12 @@
         <f>VLOOKUP(Q_start!A7,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>26052155.976207186</v>
       </c>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="L7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
       <c r="P7" s="5"/>
@@ -3130,7 +3306,7 @@
         <v>45</v>
       </c>
       <c r="B8" s="8">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="C8" s="17">
         <f t="shared" si="0"/>
@@ -3138,15 +3314,15 @@
       </c>
       <c r="D8" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A8)</f>
-        <v>17.475918265623562</v>
+        <v>0</v>
       </c>
       <c r="E8" s="15">
         <f>VLOOKUP(Medium_Capacity!A8, Medium_Capacity!A7:A24:B7:B24, 2, FALSE)</f>
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="F8" s="20">
-        <f t="shared" ref="F8:F18" si="2">E8-D8</f>
-        <v>59982.524081734373</v>
+        <f t="shared" si="1"/>
+        <v>30000</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -3159,8 +3335,12 @@
         <f>VLOOKUP(Q_start!A8,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>26052155.976207186</v>
       </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="5"/>
+      <c r="L8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
       <c r="P8" s="5"/>
@@ -3206,7 +3386,7 @@
         <v>22</v>
       </c>
       <c r="B9" s="8">
-        <v>3292700000</v>
+        <v>1646350000</v>
       </c>
       <c r="C9" s="17">
         <f t="shared" si="0"/>
@@ -3214,15 +3394,15 @@
       </c>
       <c r="D9" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A9)</f>
-        <v>813362361.42699778</v>
+        <v>974688646</v>
       </c>
       <c r="E9" s="15">
         <f>VLOOKUP(Medium_Capacity!A9, Medium_Capacity!A8:A25:B8:B25, 2, FALSE)</f>
-        <v>3292700000</v>
+        <v>1646350000</v>
       </c>
       <c r="F9" s="20">
-        <f>E9-D9</f>
-        <v>2479337638.5730023</v>
+        <f t="shared" si="1"/>
+        <v>671661354</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -3235,8 +3415,12 @@
         <f>VLOOKUP(Q_start!A9,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>7180030.7496517412</v>
       </c>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="L9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
       <c r="P9" s="5"/>
@@ -3282,7 +3466,7 @@
         <v>49</v>
       </c>
       <c r="B10" s="8">
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="C10" s="17">
         <f t="shared" si="0"/>
@@ -3290,15 +3474,15 @@
       </c>
       <c r="D10" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A10)</f>
-        <v>2202438.3659863574</v>
+        <v>12000000</v>
       </c>
       <c r="E10" s="15">
         <f>VLOOKUP(Medium_Capacity!A10, Medium_Capacity!A9:A26:B9:B26, 2, FALSE)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="F10" s="20">
-        <f t="shared" si="2"/>
-        <v>13797561.634013642</v>
+        <f t="shared" si="1"/>
+        <v>-4000000</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
@@ -3311,8 +3495,12 @@
         <f>VLOOKUP(Q_start!A10,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>7180030.7496517412</v>
       </c>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="L10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
       <c r="P10" s="5"/>
@@ -3358,7 +3546,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="8">
-        <v>121200000</v>
+        <v>60600000</v>
       </c>
       <c r="C11" s="17">
         <f t="shared" si="0"/>
@@ -3366,15 +3554,15 @@
       </c>
       <c r="D11" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A11)</f>
-        <v>15072242.234624971</v>
+        <v>116220026</v>
       </c>
       <c r="E11" s="15">
         <f>VLOOKUP(Medium_Capacity!A11, Medium_Capacity!A10:A27:B10:B27, 2, FALSE)</f>
-        <v>121200000</v>
+        <v>60600000</v>
       </c>
       <c r="F11" s="20">
-        <f t="shared" si="2"/>
-        <v>106127757.76537503</v>
+        <f t="shared" si="1"/>
+        <v>-55620026</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
@@ -3387,8 +3575,12 @@
         <f>VLOOKUP(Q_start!A11,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>7180030.7496517412</v>
       </c>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="L11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="5"/>
@@ -3434,7 +3626,7 @@
         <v>24</v>
       </c>
       <c r="B12" s="8">
-        <v>6200000</v>
+        <v>3100000</v>
       </c>
       <c r="C12" s="17">
         <f t="shared" si="0"/>
@@ -3442,15 +3634,15 @@
       </c>
       <c r="D12" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A12)</f>
-        <v>87680.677897300135</v>
+        <v>5814756</v>
       </c>
       <c r="E12" s="15">
         <f>VLOOKUP(Medium_Capacity!A12, Medium_Capacity!A11:A28:B11:B28, 2, FALSE)</f>
-        <v>6200000</v>
+        <v>3100000</v>
       </c>
       <c r="F12" s="20">
-        <f t="shared" si="2"/>
-        <v>6112319.3221026994</v>
+        <f t="shared" si="1"/>
+        <v>-2714756</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
@@ -3463,8 +3655,12 @@
         <f>VLOOKUP(Q_start!A12,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>59502552.144086249</v>
       </c>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="L12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="5"/>
@@ -3510,7 +3706,7 @@
         <v>30</v>
       </c>
       <c r="B13" s="8">
-        <v>41000000</v>
+        <v>20500000</v>
       </c>
       <c r="C13" s="17">
         <f t="shared" si="0"/>
@@ -3518,15 +3714,15 @@
       </c>
       <c r="D13" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A13)</f>
-        <v>8897918.9836929291</v>
+        <v>17896070</v>
       </c>
       <c r="E13" s="15">
         <f>VLOOKUP(Medium_Capacity!A13, Medium_Capacity!A12:A29:B12:B29, 2, FALSE)</f>
-        <v>41000000</v>
+        <v>20500000</v>
       </c>
       <c r="F13" s="20">
-        <f t="shared" si="2"/>
-        <v>32102081.016307071</v>
+        <f t="shared" si="1"/>
+        <v>2603930</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -3539,8 +3735,12 @@
         <f>VLOOKUP(Q_start!A13,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>59502552.144086249</v>
       </c>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="L13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="5"/>
@@ -3586,7 +3786,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="8">
-        <v>11600000</v>
+        <v>5800000</v>
       </c>
       <c r="C14" s="17">
         <f t="shared" si="0"/>
@@ -3594,15 +3794,15 @@
       </c>
       <c r="D14" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A14)</f>
-        <v>585672.67794888001</v>
+        <v>8000000</v>
       </c>
       <c r="E14" s="15">
         <f>VLOOKUP(Medium_Capacity!A14, Medium_Capacity!A13:A30:B13:B30, 2, FALSE)</f>
-        <v>11600000</v>
+        <v>5800000</v>
       </c>
       <c r="F14" s="20">
-        <f t="shared" si="2"/>
-        <v>11014327.322051119</v>
+        <f t="shared" si="1"/>
+        <v>-2200000</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
@@ -3613,10 +3813,14 @@
       </c>
       <c r="K14">
         <f>VLOOKUP(Q_start!A14,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
-        <v>927637.83394736843</v>
-      </c>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+        <v>927637.83394736797</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="5"/>
@@ -3662,7 +3866,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="8">
-        <v>233200000</v>
+        <v>116600000</v>
       </c>
       <c r="C15" s="17">
         <f t="shared" si="0"/>
@@ -3670,15 +3874,15 @@
       </c>
       <c r="D15" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A15)</f>
-        <v>70514508.456252947</v>
+        <v>173915770</v>
       </c>
       <c r="E15" s="15">
         <f>VLOOKUP(Medium_Capacity!A15, Medium_Capacity!A14:A31:B14:B31, 2, FALSE)</f>
-        <v>233200000</v>
+        <v>116600000</v>
       </c>
       <c r="F15" s="20">
-        <f t="shared" si="2"/>
-        <v>162685491.54374707</v>
+        <f t="shared" si="1"/>
+        <v>-57315770</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
@@ -3689,10 +3893,14 @@
       </c>
       <c r="K15">
         <f>VLOOKUP(Q_start!A15,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
-        <v>927637.83394736843</v>
-      </c>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+        <v>927637.83394736797</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="5"/>
@@ -3738,7 +3946,7 @@
         <v>33</v>
       </c>
       <c r="B16" s="8">
-        <v>209200000</v>
+        <v>104600000</v>
       </c>
       <c r="C16" s="17">
         <f t="shared" si="0"/>
@@ -3746,15 +3954,15 @@
       </c>
       <c r="D16" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A16)</f>
-        <v>34360914.23466716</v>
+        <v>209171984</v>
       </c>
       <c r="E16" s="15">
         <f>VLOOKUP(Medium_Capacity!A16, Medium_Capacity!A15:A32:B15:B32, 2, FALSE)</f>
-        <v>209200000</v>
+        <v>104600000</v>
       </c>
       <c r="F16" s="20">
-        <f t="shared" si="2"/>
-        <v>174839085.76533285</v>
+        <f t="shared" si="1"/>
+        <v>-104571984</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
@@ -3765,10 +3973,14 @@
       </c>
       <c r="K16">
         <f>VLOOKUP(Q_start!A16,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
-        <v>927637.83394736843</v>
-      </c>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+        <v>927637.83394736797</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="5"/>
@@ -3814,7 +4026,7 @@
         <v>23</v>
       </c>
       <c r="B17" s="8">
-        <v>1938750500</v>
+        <v>969375250</v>
       </c>
       <c r="C17" s="17">
         <f t="shared" si="0"/>
@@ -3822,15 +4034,15 @@
       </c>
       <c r="D17" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A17)</f>
-        <v>1066483631.1790735</v>
+        <v>975046998</v>
       </c>
       <c r="E17" s="15">
         <f>VLOOKUP(Medium_Capacity!A17, Medium_Capacity!A16:A33:B16:B33, 2, FALSE)</f>
-        <v>1938750500</v>
+        <v>969375250</v>
       </c>
       <c r="F17" s="20">
-        <f t="shared" si="2"/>
-        <v>872266868.82092655</v>
+        <f>E17-D17</f>
+        <v>-5671748</v>
       </c>
       <c r="J17">
         <f>VLOOKUP(Q_start!B17,Medium_Capacity!$B$30:$C$46,2)</f>
@@ -3840,7 +4052,12 @@
         <f>VLOOKUP(Q_start!A17,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>83779046.847486719</v>
       </c>
-      <c r="M17" s="5"/>
+      <c r="L17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
@@ -3886,7 +4103,7 @@
         <v>35</v>
       </c>
       <c r="B18" s="8">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="C18" s="17">
         <f t="shared" si="0"/>
@@ -3894,15 +4111,15 @@
       </c>
       <c r="D18" s="16">
         <f>SUMIFS(Q_start!E:E, Q_start!B:B, Medium_Capacity!A18)</f>
-        <v>5962.0322529060686</v>
+        <v>0</v>
       </c>
       <c r="E18" s="15">
         <f>VLOOKUP(Medium_Capacity!A18, Medium_Capacity!A17:A34:B17:B34, 2, FALSE)</f>
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="F18" s="20">
-        <f t="shared" si="2"/>
-        <v>994037.96774709388</v>
+        <f t="shared" si="1"/>
+        <v>500000</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -3915,8 +4132,12 @@
         <f>VLOOKUP(Q_start!A18,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>83779046.847486719</v>
       </c>
-      <c r="L18" s="8"/>
-      <c r="M18" s="5"/>
+      <c r="L18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
       <c r="P18" s="5"/>
@@ -3974,11 +4195,17 @@
         <f>VLOOKUP(Q_start!A19,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>83779046.847486719</v>
       </c>
+      <c r="L19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M19" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B20" s="9">
         <f>SUM(B2:B18)</f>
-        <v>6369710500</v>
+        <v>3184855250</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
@@ -3994,6 +4221,12 @@
       <c r="K20">
         <f>VLOOKUP(Q_start!A20,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>83779046.847486719</v>
+      </c>
+      <c r="L20" t="s">
+        <v>32</v>
+      </c>
+      <c r="M20" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
@@ -4013,6 +4246,12 @@
         <f>VLOOKUP(Q_start!A21,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
+      <c r="L21" t="s">
+        <v>34</v>
+      </c>
+      <c r="M21" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B22" s="7"/>
@@ -4031,6 +4270,12 @@
         <f>VLOOKUP(Q_start!A22,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
+      <c r="L22" t="s">
+        <v>34</v>
+      </c>
+      <c r="M22" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B23" s="8"/>
@@ -4049,7 +4294,12 @@
         <f>VLOOKUP(Q_start!A23,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L23" s="8"/>
+      <c r="L23" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M23" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="24" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B24" s="8"/>
@@ -4068,7 +4318,12 @@
         <f>VLOOKUP(Q_start!A24,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L24" s="8"/>
+      <c r="L24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M24" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="25" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B25" s="8"/>
@@ -4087,7 +4342,12 @@
         <f>VLOOKUP(Q_start!A25,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L25" s="8"/>
+      <c r="L25" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M25" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B26" s="8"/>
@@ -4106,7 +4366,12 @@
         <f>VLOOKUP(Q_start!A26,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L26" s="8"/>
+      <c r="L26" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M26" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="27" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B27" s="8"/>
@@ -4125,7 +4390,12 @@
         <f>VLOOKUP(Q_start!A27,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L27" s="8"/>
+      <c r="L27" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M27" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
       <c r="E28" s="8"/>
@@ -4141,7 +4411,12 @@
         <f>VLOOKUP(Q_start!A28,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>438402962.04456699</v>
       </c>
-      <c r="L28" s="8"/>
+      <c r="L28" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M28" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="29" spans="1:52" x14ac:dyDescent="0.25">
       <c r="E29" s="8"/>
@@ -4157,7 +4432,12 @@
         <f>VLOOKUP(Q_start!A29,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>6404901.9598684218</v>
       </c>
-      <c r="L29" s="8"/>
+      <c r="L29" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M29" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
@@ -4179,7 +4459,12 @@
         <f>VLOOKUP(Q_start!A30,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>6404901.9598684218</v>
       </c>
-      <c r="L30" s="8"/>
+      <c r="L30" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M30" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
@@ -4201,7 +4486,12 @@
         <f>VLOOKUP(Q_start!A31,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>6404901.9598684218</v>
       </c>
-      <c r="L31" s="8"/>
+      <c r="L31" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M31" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="32" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
@@ -4223,9 +4513,14 @@
         <f>VLOOKUP(Q_start!A32,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>243482508.59073868</v>
       </c>
-      <c r="L32" s="8"/>
-    </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L32" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>36</v>
       </c>
@@ -4245,9 +4540,14 @@
         <f>VLOOKUP(Q_start!A33,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>243482508.59073868</v>
       </c>
-      <c r="L33" s="8"/>
-    </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L33" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M33" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>47</v>
       </c>
@@ -4267,9 +4567,14 @@
         <f>VLOOKUP(Q_start!A34,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>243482508.59073868</v>
       </c>
-      <c r="L34" s="8"/>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L34" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M34" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>26</v>
       </c>
@@ -4289,9 +4594,14 @@
         <f>VLOOKUP(Q_start!A35,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>62054151.5187333</v>
       </c>
-      <c r="L35" s="8"/>
-    </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L35" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="M35" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>45</v>
       </c>
@@ -4311,9 +4621,14 @@
         <f>VLOOKUP(Q_start!A36,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>62054151.5187333</v>
       </c>
-      <c r="L36" s="8"/>
-    </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L36" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="M36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>22</v>
       </c>
@@ -4333,9 +4648,14 @@
         <f>VLOOKUP(Q_start!A37,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>5826576.9305263162</v>
       </c>
-      <c r="L37" s="8"/>
-    </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L37" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M37" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>49</v>
       </c>
@@ -4355,9 +4675,14 @@
         <f>VLOOKUP(Q_start!A38,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>252782013.30394739</v>
       </c>
-      <c r="L38" s="8"/>
-    </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L38" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M38" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -4377,9 +4702,14 @@
         <f>VLOOKUP(Q_start!A39,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>252782013.30394739</v>
       </c>
-      <c r="L39" s="8"/>
-    </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L39" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M39" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>24</v>
       </c>
@@ -4399,9 +4729,14 @@
         <f>VLOOKUP(Q_start!A40,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>252782013.30394739</v>
       </c>
-      <c r="L40" s="8"/>
-    </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L40" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>30</v>
       </c>
@@ -4421,9 +4756,14 @@
         <f>VLOOKUP(Q_start!A41,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>252782013.30394739</v>
       </c>
-      <c r="L41" s="8"/>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L41" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>37</v>
       </c>
@@ -4443,9 +4783,14 @@
         <f>VLOOKUP(Q_start!A42,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>252782013.30394739</v>
       </c>
-      <c r="L42" s="8"/>
-    </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L42" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>20</v>
       </c>
@@ -4465,9 +4810,14 @@
         <f>VLOOKUP(Q_start!A43,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="L43" s="8"/>
-    </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L43" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>33</v>
       </c>
@@ -4487,9 +4837,14 @@
         <f>VLOOKUP(Q_start!A44,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>18988209.721337222</v>
       </c>
-      <c r="L44" s="8"/>
-    </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L44" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="M44" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>23</v>
       </c>
@@ -4504,8 +4859,14 @@
         <f>VLOOKUP(Q_start!A45,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>18988209.721337222</v>
       </c>
-    </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L45" t="s">
+        <v>9</v>
+      </c>
+      <c r="M45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>35</v>
       </c>
@@ -4520,8 +4881,14 @@
         <f>VLOOKUP(Q_start!A46,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>18988209.721337222</v>
       </c>
-    </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L46" t="s">
+        <v>9</v>
+      </c>
+      <c r="M46" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="J47">
         <f>VLOOKUP(Q_start!B47,Medium_Capacity!$B$30:$C$46,2)</f>
         <v>0.30437026926105981</v>
@@ -4530,8 +4897,14 @@
         <f>VLOOKUP(Q_start!A47,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>142479003.36778629</v>
       </c>
-    </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L47" t="s">
+        <v>10</v>
+      </c>
+      <c r="M47" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="J48">
@@ -4542,8 +4915,14 @@
         <f>VLOOKUP(Q_start!A48,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>142479003.36778629</v>
       </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="L48" t="s">
+        <v>10</v>
+      </c>
+      <c r="M48" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>19</v>
       </c>
@@ -4559,8 +4938,14 @@
         <f>VLOOKUP(Q_start!A49,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>142479003.36778629</v>
       </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="L49" t="s">
+        <v>10</v>
+      </c>
+      <c r="M49" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>25</v>
       </c>
@@ -4576,8 +4961,14 @@
         <f>VLOOKUP(Q_start!A50,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>160800233.02991807</v>
       </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="L50" t="s">
+        <v>13</v>
+      </c>
+      <c r="M50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>21</v>
       </c>
@@ -4593,8 +4984,14 @@
         <f>VLOOKUP(Q_start!A51,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>160800233.02991807</v>
       </c>
-    </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="L51" t="s">
+        <v>13</v>
+      </c>
+      <c r="M51" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>39</v>
       </c>
@@ -4610,8 +5007,14 @@
         <f>VLOOKUP(Q_start!A52,Medium_Capacity!$B$49:$C$65,2, FALSE)</f>
         <v>160800233.02991807</v>
       </c>
-    </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="L52" t="s">
+        <v>13</v>
+      </c>
+      <c r="M52" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>27</v>
       </c>
@@ -4620,7 +5023,7 @@
       </c>
       <c r="D53" s="2"/>
     </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>41</v>
       </c>
@@ -4629,7 +5032,7 @@
       </c>
       <c r="D54" s="2"/>
     </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>42</v>
       </c>
@@ -4638,7 +5041,7 @@
       </c>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>43</v>
       </c>
@@ -4646,7 +5049,7 @@
         <v>5826576.9305263162</v>
       </c>
     </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>29</v>
       </c>
@@ -4654,7 +5057,7 @@
         <v>252782013.30394739</v>
       </c>
     </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>44</v>
       </c>
@@ -4662,7 +5065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>32</v>
       </c>
@@ -4670,7 +5073,7 @@
         <v>83779046.847486719</v>
       </c>
     </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>34</v>
       </c>
@@ -4678,7 +5081,7 @@
         <v>438402962.04456699</v>
       </c>
     </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>9</v>
       </c>
@@ -4686,7 +5089,7 @@
         <v>18988209.721337222</v>
       </c>
     </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>40</v>
       </c>
@@ -4694,15 +5097,15 @@
         <v>59502552.144086249</v>
       </c>
     </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>7</v>
       </c>
       <c r="C63">
-        <v>927637.83394736843</v>
-      </c>
-    </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.25">
+        <v>927637.83394736797</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>10</v>
       </c>

</xml_diff>